<commit_message>
Save as csv & add metric code
</commit_message>
<xml_diff>
--- a/casebase/statistics/rerord.xlsx
+++ b/casebase/statistics/rerord.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\0_code\block-gml-casebase\casebase\record_temp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\0_codes\block-gml-casebase\casebase\statistics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2978715-DFCA-4A56-86AB-89C763AB269D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2978715-DFCA-4A56-86AB-89C763AB269D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9564" xr2:uid="{7E148D5C-DE84-49D0-B495-48D3DA96E5A6}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{7E148D5C-DE84-49D0-B495-48D3DA96E5A6}"/>
   </bookViews>
   <sheets>
     <sheet name="Block" sheetId="3" r:id="rId1"/>
@@ -897,53 +897,50 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1264,23 +1261,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82B6020B-322E-40F5-A134-4E53684558CD}">
   <dimension ref="A1:N35"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17" style="1" customWidth="1"/>
     <col min="2" max="2" width="14.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="13.44140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="10.88671875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="13.4140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10.9140625" style="1" customWidth="1"/>
     <col min="5" max="5" width="9.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.109375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="14.88671875" style="1" customWidth="1"/>
-    <col min="8" max="9" width="9.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.08203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="14.9140625" style="1" customWidth="1"/>
+    <col min="8" max="9" width="9.08203125" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="12" width="9" style="1"/>
-    <col min="13" max="13" width="11.21875" style="1" customWidth="1"/>
-    <col min="14" max="14" width="12.109375" style="1" customWidth="1"/>
+    <col min="13" max="13" width="11.25" style="1" customWidth="1"/>
+    <col min="14" max="14" width="12.08203125" style="1" customWidth="1"/>
     <col min="15" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="41.4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" ht="42" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>11</v>
       </c>
@@ -1318,7 +1315,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>14</v>
       </c>
@@ -1358,7 +1355,7 @@
         <v>79550</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>24</v>
       </c>
@@ -1390,7 +1387,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>17</v>
       </c>
@@ -1422,7 +1419,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>32</v>
       </c>
@@ -1451,7 +1448,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>16</v>
       </c>
@@ -1483,7 +1480,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>49</v>
       </c>
@@ -1515,7 +1512,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>47</v>
       </c>
@@ -1544,7 +1541,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>52</v>
       </c>
@@ -1573,7 +1570,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="10" spans="1:14" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
         <v>53</v>
       </c>
@@ -1602,7 +1599,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>57</v>
       </c>
@@ -1631,7 +1628,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>60</v>
       </c>
@@ -1663,7 +1660,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="13" spans="1:14" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
         <v>72</v>
       </c>
@@ -1695,7 +1692,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>51</v>
       </c>
@@ -1727,7 +1724,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>62</v>
       </c>
@@ -1759,7 +1756,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>103</v>
       </c>
@@ -1788,7 +1785,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>104</v>
       </c>
@@ -1817,7 +1814,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>105</v>
       </c>
@@ -1846,7 +1843,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>112</v>
       </c>
@@ -1875,7 +1872,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>113</v>
       </c>
@@ -1904,7 +1901,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>120</v>
       </c>
@@ -1933,7 +1930,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>127</v>
       </c>
@@ -1962,7 +1959,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>128</v>
       </c>
@@ -1991,7 +1988,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>132</v>
       </c>
@@ -2020,7 +2017,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>138</v>
       </c>
@@ -2050,7 +2047,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>140</v>
       </c>
@@ -2079,7 +2076,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
         <v>155</v>
       </c>
@@ -2108,7 +2105,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="28" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>149</v>
       </c>
@@ -2138,7 +2135,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>152</v>
       </c>
@@ -2167,7 +2164,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="8" t="s">
         <v>156</v>
       </c>
@@ -2197,7 +2194,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>164</v>
       </c>
@@ -2226,7 +2223,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
         <v>173</v>
       </c>
@@ -2255,7 +2252,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>178</v>
       </c>
@@ -2287,7 +2284,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>182</v>
       </c>
@@ -2316,7 +2313,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>187</v>
       </c>
@@ -2355,28 +2352,28 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BD8883F-BF25-46E4-9E09-E50E86F863DC}">
   <dimension ref="A1:Y27"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.77734375" style="3" customWidth="1"/>
+    <col min="1" max="1" width="14.75" style="3" customWidth="1"/>
     <col min="2" max="2" width="57.6640625" style="3" customWidth="1"/>
     <col min="3" max="3" width="9" style="3" customWidth="1"/>
-    <col min="4" max="4" width="10.88671875" style="3" customWidth="1"/>
+    <col min="4" max="4" width="10.9140625" style="3" customWidth="1"/>
     <col min="5" max="5" width="11.33203125" style="3" customWidth="1"/>
-    <col min="6" max="6" width="8.109375" style="3" customWidth="1"/>
-    <col min="7" max="7" width="14.109375" style="3" customWidth="1"/>
-    <col min="8" max="8" width="10.44140625" style="3" customWidth="1"/>
-    <col min="9" max="9" width="11.77734375" style="3" customWidth="1"/>
-    <col min="10" max="10" width="14.109375" style="3" customWidth="1"/>
-    <col min="11" max="11" width="11.77734375" style="3" customWidth="1"/>
-    <col min="12" max="12" width="23.88671875" style="3" customWidth="1"/>
+    <col min="6" max="6" width="8.08203125" style="3" customWidth="1"/>
+    <col min="7" max="7" width="14.08203125" style="3" customWidth="1"/>
+    <col min="8" max="8" width="10.4140625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="11.75" style="3" customWidth="1"/>
+    <col min="10" max="10" width="14.08203125" style="3" customWidth="1"/>
+    <col min="11" max="11" width="11.75" style="3" customWidth="1"/>
+    <col min="12" max="12" width="23.9140625" style="3" customWidth="1"/>
     <col min="13" max="15" width="9" style="3"/>
     <col min="16" max="16" width="11.6640625" style="3" customWidth="1"/>
-    <col min="17" max="17" width="12.5546875" style="3" customWidth="1"/>
-    <col min="18" max="18" width="11.109375" style="3" customWidth="1"/>
+    <col min="17" max="17" width="12.58203125" style="3" customWidth="1"/>
+    <col min="18" max="18" width="11.08203125" style="3" customWidth="1"/>
     <col min="19" max="16384" width="9" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="41.4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" ht="42" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
@@ -2429,7 +2426,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" ht="28" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -2489,7 +2486,7 @@
       <c r="X2" s="1"/>
       <c r="Y2" s="1"/>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>17</v>
       </c>
@@ -2528,7 +2525,7 @@
       </c>
       <c r="X3" s="7"/>
     </row>
-    <row r="4" spans="1:25" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" ht="28" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>60</v>
       </c>
@@ -2563,7 +2560,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" ht="28" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>62</v>
       </c>
@@ -2598,7 +2595,7 @@
         <v>6.6</v>
       </c>
     </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>51</v>
       </c>
@@ -2636,7 +2633,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="7" spans="1:25" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" ht="28" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>46</v>
       </c>
@@ -2674,7 +2671,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>103</v>
       </c>
@@ -2712,7 +2709,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="41.4" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>104</v>
       </c>
@@ -2747,7 +2744,7 @@
         <v>1.43</v>
       </c>
     </row>
-    <row r="10" spans="1:25" ht="41.4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" ht="28" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>105</v>
       </c>
@@ -2782,7 +2779,7 @@
         <v>0.11</v>
       </c>
     </row>
-    <row r="11" spans="1:25" ht="41.4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" ht="28" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>112</v>
       </c>
@@ -2823,7 +2820,7 @@
       <c r="S11" s="1"/>
       <c r="T11" s="1"/>
     </row>
-    <row r="12" spans="1:25" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" ht="40.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>72</v>
       </c>
@@ -2861,7 +2858,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" spans="1:25" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" ht="42.65" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>113</v>
       </c>
@@ -2896,7 +2893,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>120</v>
       </c>
@@ -2934,7 +2931,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="15" spans="1:25" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:25" ht="28" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>122</v>
       </c>
@@ -2969,7 +2966,7 @@
         <v>7.52</v>
       </c>
     </row>
-    <row r="16" spans="1:25" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>128</v>
       </c>
@@ -3004,7 +3001,7 @@
         <v>7.87</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" ht="28" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>132</v>
       </c>
@@ -3039,7 +3036,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>140</v>
       </c>
@@ -3074,7 +3071,7 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>145</v>
       </c>
@@ -3099,7 +3096,7 @@
       <c r="H19" s="3">
         <v>7796212</v>
       </c>
-      <c r="I19" s="13">
+      <c r="I19" s="1">
         <v>31256</v>
       </c>
       <c r="J19" s="3">
@@ -3109,7 +3106,7 @@
         <v>0.26</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>147</v>
       </c>
@@ -3144,7 +3141,7 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="21" spans="1:12" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" ht="28" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
         <v>156</v>
       </c>
@@ -3169,7 +3166,7 @@
       <c r="H21" s="6">
         <v>59562180</v>
       </c>
-      <c r="I21" s="14">
+      <c r="I21" s="13">
         <v>4490</v>
       </c>
       <c r="J21" s="6">
@@ -3182,7 +3179,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="41.4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" ht="28" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>169</v>
       </c>
@@ -3217,7 +3214,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="23" spans="1:12" ht="41.4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" ht="28" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>173</v>
       </c>
@@ -3252,7 +3249,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="24" spans="1:12" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" ht="28" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>182</v>
       </c>
@@ -3290,7 +3287,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" ht="28" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>178</v>
       </c>
@@ -3328,45 +3325,45 @@
         <v>186</v>
       </c>
     </row>
-    <row r="26" spans="1:12" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="A26" s="15" t="s">
+    <row r="26" spans="1:12" ht="28" x14ac:dyDescent="0.3">
+      <c r="A26" s="14" t="s">
         <v>187</v>
       </c>
-      <c r="B26" s="15" t="s">
+      <c r="B26" s="14" t="s">
         <v>185</v>
       </c>
-      <c r="C26" s="15">
+      <c r="C26" s="14">
         <v>1</v>
       </c>
-      <c r="D26" s="15">
+      <c r="D26" s="14">
         <v>20260203</v>
       </c>
-      <c r="E26" s="15">
+      <c r="E26" s="14">
         <v>20260508</v>
       </c>
-      <c r="F26" s="15" t="s">
+      <c r="F26" s="14" t="s">
         <v>184</v>
       </c>
-      <c r="G26" s="15">
+      <c r="G26" s="14">
         <v>153114</v>
       </c>
-      <c r="H26" s="15">
+      <c r="H26" s="14">
         <v>1711200</v>
       </c>
       <c r="I26" s="3">
         <v>2154</v>
       </c>
-      <c r="J26" s="15">
+      <c r="J26" s="14">
         <v>108650</v>
       </c>
-      <c r="K26" s="15">
+      <c r="K26" s="14">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="L26" s="15" t="s">
+      <c r="L26" s="14" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="27" spans="1:12" s="15" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="1:12" s="14" customFormat="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
@@ -3382,28 +3379,28 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{830BA63A-35BF-480A-BCDB-E5D49BE645A6}">
   <dimension ref="A1:S20"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.77734375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="76.88671875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="9.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.75" style="3" customWidth="1"/>
+    <col min="2" max="2" width="76.9140625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="9.08203125" style="3" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.6640625" style="3" customWidth="1"/>
     <col min="5" max="5" width="9.6640625" style="3" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9" style="3"/>
-    <col min="7" max="7" width="9.109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.21875" style="3" customWidth="1"/>
-    <col min="9" max="9" width="9.109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.77734375" style="3" customWidth="1"/>
-    <col min="11" max="11" width="16.77734375" style="3" customWidth="1"/>
-    <col min="12" max="12" width="26.109375" style="3" customWidth="1"/>
+    <col min="7" max="7" width="9.08203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.25" style="3" customWidth="1"/>
+    <col min="9" max="9" width="9.08203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.75" style="3" customWidth="1"/>
+    <col min="11" max="11" width="16.75" style="3" customWidth="1"/>
+    <col min="12" max="12" width="26.08203125" style="3" customWidth="1"/>
     <col min="13" max="15" width="9" style="3"/>
-    <col min="16" max="16" width="11.44140625" style="3" customWidth="1"/>
-    <col min="17" max="17" width="13.109375" style="3" customWidth="1"/>
-    <col min="18" max="19" width="9.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.4140625" style="3" customWidth="1"/>
+    <col min="17" max="17" width="13.08203125" style="3" customWidth="1"/>
+    <col min="18" max="19" width="9.08203125" style="3" bestFit="1" customWidth="1"/>
     <col min="20" max="16384" width="9" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" ht="28" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
@@ -3456,7 +3453,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -3511,7 +3508,7 @@
         <v>86.720000000000013</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>24</v>
       </c>
@@ -3546,7 +3543,7 @@
         <v>11.1</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" ht="28" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>17</v>
       </c>
@@ -3581,7 +3578,7 @@
         <v>1.01</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" ht="28" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>32</v>
       </c>
@@ -3619,7 +3616,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" ht="28" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>43</v>
       </c>
@@ -3654,7 +3651,7 @@
         <v>7.41</v>
       </c>
     </row>
-    <row r="7" spans="1:19" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>46</v>
       </c>
@@ -3689,7 +3686,7 @@
         <v>1.03</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="69" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" ht="70" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>47</v>
       </c>
@@ -3724,7 +3721,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>52</v>
       </c>
@@ -3759,7 +3756,7 @@
         <v>0.78</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="110.4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" ht="98" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
         <v>53</v>
       </c>
@@ -3797,7 +3794,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>57</v>
       </c>
@@ -3832,7 +3829,7 @@
         <v>4.72</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>60</v>
       </c>
@@ -3867,7 +3864,7 @@
         <v>3.69</v>
       </c>
     </row>
-    <row r="13" spans="1:19" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" ht="28" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>62</v>
       </c>
@@ -3905,7 +3902,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="14" spans="1:19" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:19" ht="28" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
         <v>72</v>
       </c>
@@ -3943,7 +3940,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="15" spans="1:19" s="11" customFormat="1" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:19" s="11" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>51</v>
       </c>
@@ -3978,7 +3975,7 @@
         <v>1.04</v>
       </c>
     </row>
-    <row r="16" spans="1:19" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:19" ht="28" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
         <v>138</v>
       </c>
@@ -4016,7 +4013,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>149</v>
       </c>
@@ -4048,7 +4045,7 @@
         <v>5.97</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>152</v>
       </c>
@@ -4080,7 +4077,7 @@
         <v>3.29</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" ht="28" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>164</v>
       </c>
@@ -4115,7 +4112,7 @@
         <v>4.68</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" ht="28" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>178</v>
       </c>

</xml_diff>